<commit_message>
Fix Flow State publishable result content statuses
</commit_message>
<xml_diff>
--- a/content/assessment-packages/flow-state/sonartra_reader_first_import_schema_FLOW_STATE_EXAMPLE.xlsx
+++ b/content/assessment-packages/flow-state/sonartra_reader_first_import_schema_FLOW_STATE_EXAMPLE.xlsx
@@ -19191,19 +19191,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K2"/>
-  <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="28.83203125" customWidth="1"/>
-    <col min="5" max="5" width="58.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="34.83203125" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" customWidth="1"/>
-    <col min="9" max="9" width="58.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20259,14 +20246,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F25"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="58.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20778,16 +20757,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H97"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="58.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23321,15 +23290,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G97"/>
-  <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="38.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -25736,7 +25696,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O2" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P2" t="str">
         <v>flow-state::deep_focus_creative_movement_physical_rhythm_social_exchange::concentrated</v>
@@ -25786,7 +25746,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O3" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P3" t="str">
         <v>flow-state::deep_focus_creative_movement_physical_rhythm_social_exchange::paired</v>
@@ -25836,7 +25796,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O4" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P4" t="str">
         <v>flow-state::deep_focus_creative_movement_physical_rhythm_social_exchange::graduated</v>
@@ -25886,7 +25846,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O5" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P5" t="str">
         <v>flow-state::deep_focus_creative_movement_physical_rhythm_social_exchange::balanced</v>
@@ -25936,7 +25896,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O6" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P6" t="str">
         <v>flow-state::deep_focus_creative_movement_social_exchange_physical_rhythm::concentrated</v>
@@ -25986,7 +25946,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O7" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P7" t="str">
         <v>flow-state::deep_focus_creative_movement_social_exchange_physical_rhythm::paired</v>
@@ -26036,7 +25996,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O8" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P8" t="str">
         <v>flow-state::deep_focus_creative_movement_social_exchange_physical_rhythm::graduated</v>
@@ -26086,7 +26046,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O9" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P9" t="str">
         <v>flow-state::deep_focus_creative_movement_social_exchange_physical_rhythm::balanced</v>
@@ -26136,7 +26096,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O10" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P10" t="str">
         <v>flow-state::deep_focus_physical_rhythm_creative_movement_social_exchange::concentrated</v>
@@ -26186,7 +26146,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O11" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P11" t="str">
         <v>flow-state::deep_focus_physical_rhythm_creative_movement_social_exchange::paired</v>
@@ -26236,7 +26196,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O12" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P12" t="str">
         <v>flow-state::deep_focus_physical_rhythm_creative_movement_social_exchange::graduated</v>
@@ -26286,7 +26246,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O13" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P13" t="str">
         <v>flow-state::deep_focus_physical_rhythm_creative_movement_social_exchange::balanced</v>
@@ -26336,7 +26296,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O14" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P14" t="str">
         <v>flow-state::deep_focus_physical_rhythm_social_exchange_creative_movement::concentrated</v>
@@ -26386,7 +26346,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O15" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P15" t="str">
         <v>flow-state::deep_focus_physical_rhythm_social_exchange_creative_movement::paired</v>
@@ -26436,7 +26396,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O16" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P16" t="str">
         <v>flow-state::deep_focus_physical_rhythm_social_exchange_creative_movement::graduated</v>
@@ -26486,7 +26446,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O17" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P17" t="str">
         <v>flow-state::deep_focus_physical_rhythm_social_exchange_creative_movement::balanced</v>
@@ -26536,7 +26496,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O18" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P18" t="str">
         <v>flow-state::deep_focus_social_exchange_creative_movement_physical_rhythm::concentrated</v>
@@ -26586,7 +26546,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O19" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P19" t="str">
         <v>flow-state::deep_focus_social_exchange_creative_movement_physical_rhythm::paired</v>
@@ -26636,7 +26596,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O20" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P20" t="str">
         <v>flow-state::deep_focus_social_exchange_creative_movement_physical_rhythm::graduated</v>
@@ -26686,7 +26646,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O21" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P21" t="str">
         <v>flow-state::deep_focus_social_exchange_creative_movement_physical_rhythm::balanced</v>
@@ -26736,7 +26696,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O22" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P22" t="str">
         <v>flow-state::deep_focus_social_exchange_physical_rhythm_creative_movement::concentrated</v>
@@ -26786,7 +26746,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O23" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P23" t="str">
         <v>flow-state::deep_focus_social_exchange_physical_rhythm_creative_movement::paired</v>
@@ -26836,7 +26796,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O24" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P24" t="str">
         <v>flow-state::deep_focus_social_exchange_physical_rhythm_creative_movement::graduated</v>
@@ -26886,7 +26846,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O25" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P25" t="str">
         <v>flow-state::deep_focus_social_exchange_physical_rhythm_creative_movement::balanced</v>
@@ -26936,7 +26896,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O26" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P26" t="str">
         <v>flow-state::creative_movement_deep_focus_physical_rhythm_social_exchange::concentrated</v>
@@ -26986,7 +26946,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O27" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P27" t="str">
         <v>flow-state::creative_movement_deep_focus_physical_rhythm_social_exchange::paired</v>
@@ -27036,7 +26996,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O28" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P28" t="str">
         <v>flow-state::creative_movement_deep_focus_physical_rhythm_social_exchange::graduated</v>
@@ -27086,7 +27046,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O29" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P29" t="str">
         <v>flow-state::creative_movement_deep_focus_physical_rhythm_social_exchange::balanced</v>
@@ -27136,7 +27096,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O30" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P30" t="str">
         <v>flow-state::creative_movement_deep_focus_social_exchange_physical_rhythm::concentrated</v>
@@ -27186,7 +27146,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O31" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P31" t="str">
         <v>flow-state::creative_movement_deep_focus_social_exchange_physical_rhythm::paired</v>
@@ -27236,7 +27196,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O32" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P32" t="str">
         <v>flow-state::creative_movement_deep_focus_social_exchange_physical_rhythm::graduated</v>
@@ -27286,7 +27246,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O33" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P33" t="str">
         <v>flow-state::creative_movement_deep_focus_social_exchange_physical_rhythm::balanced</v>
@@ -27336,7 +27296,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O34" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P34" t="str">
         <v>flow-state::creative_movement_physical_rhythm_deep_focus_social_exchange::concentrated</v>
@@ -27386,7 +27346,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O35" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P35" t="str">
         <v>flow-state::creative_movement_physical_rhythm_deep_focus_social_exchange::paired</v>
@@ -27436,7 +27396,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O36" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P36" t="str">
         <v>flow-state::creative_movement_physical_rhythm_deep_focus_social_exchange::graduated</v>
@@ -27486,7 +27446,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O37" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P37" t="str">
         <v>flow-state::creative_movement_physical_rhythm_deep_focus_social_exchange::balanced</v>
@@ -27536,7 +27496,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O38" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P38" t="str">
         <v>flow-state::creative_movement_physical_rhythm_social_exchange_deep_focus::concentrated</v>
@@ -27586,7 +27546,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O39" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P39" t="str">
         <v>flow-state::creative_movement_physical_rhythm_social_exchange_deep_focus::paired</v>
@@ -27636,7 +27596,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O40" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P40" t="str">
         <v>flow-state::creative_movement_physical_rhythm_social_exchange_deep_focus::graduated</v>
@@ -27686,7 +27646,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O41" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P41" t="str">
         <v>flow-state::creative_movement_physical_rhythm_social_exchange_deep_focus::balanced</v>
@@ -27736,7 +27696,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O42" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P42" t="str">
         <v>flow-state::creative_movement_social_exchange_deep_focus_physical_rhythm::concentrated</v>
@@ -27786,7 +27746,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O43" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P43" t="str">
         <v>flow-state::creative_movement_social_exchange_deep_focus_physical_rhythm::paired</v>
@@ -27836,7 +27796,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O44" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P44" t="str">
         <v>flow-state::creative_movement_social_exchange_deep_focus_physical_rhythm::graduated</v>
@@ -27886,7 +27846,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O45" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P45" t="str">
         <v>flow-state::creative_movement_social_exchange_deep_focus_physical_rhythm::balanced</v>
@@ -27936,7 +27896,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O46" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P46" t="str">
         <v>flow-state::creative_movement_social_exchange_physical_rhythm_deep_focus::concentrated</v>
@@ -27986,7 +27946,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O47" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P47" t="str">
         <v>flow-state::creative_movement_social_exchange_physical_rhythm_deep_focus::paired</v>
@@ -28036,7 +27996,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O48" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P48" t="str">
         <v>flow-state::creative_movement_social_exchange_physical_rhythm_deep_focus::graduated</v>
@@ -28086,7 +28046,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O49" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P49" t="str">
         <v>flow-state::creative_movement_social_exchange_physical_rhythm_deep_focus::balanced</v>
@@ -28136,7 +28096,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O50" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P50" t="str">
         <v>flow-state::physical_rhythm_deep_focus_creative_movement_social_exchange::concentrated</v>
@@ -28186,7 +28146,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O51" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P51" t="str">
         <v>flow-state::physical_rhythm_deep_focus_creative_movement_social_exchange::paired</v>
@@ -28236,7 +28196,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O52" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P52" t="str">
         <v>flow-state::physical_rhythm_deep_focus_creative_movement_social_exchange::graduated</v>
@@ -28286,7 +28246,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O53" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P53" t="str">
         <v>flow-state::physical_rhythm_deep_focus_creative_movement_social_exchange::balanced</v>
@@ -28336,7 +28296,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O54" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P54" t="str">
         <v>flow-state::physical_rhythm_deep_focus_social_exchange_creative_movement::concentrated</v>
@@ -28386,7 +28346,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O55" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P55" t="str">
         <v>flow-state::physical_rhythm_deep_focus_social_exchange_creative_movement::paired</v>
@@ -28436,7 +28396,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O56" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P56" t="str">
         <v>flow-state::physical_rhythm_deep_focus_social_exchange_creative_movement::graduated</v>
@@ -28486,7 +28446,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O57" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P57" t="str">
         <v>flow-state::physical_rhythm_deep_focus_social_exchange_creative_movement::balanced</v>
@@ -28536,7 +28496,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O58" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P58" t="str">
         <v>flow-state::physical_rhythm_creative_movement_deep_focus_social_exchange::concentrated</v>
@@ -28586,7 +28546,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O59" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P59" t="str">
         <v>flow-state::physical_rhythm_creative_movement_deep_focus_social_exchange::paired</v>
@@ -28636,7 +28596,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O60" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P60" t="str">
         <v>flow-state::physical_rhythm_creative_movement_deep_focus_social_exchange::graduated</v>
@@ -28686,7 +28646,7 @@
         <v>What to use deliberately: conversation and feedback before the work becomes too private.</v>
       </c>
       <c r="O61" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P61" t="str">
         <v>flow-state::physical_rhythm_creative_movement_deep_focus_social_exchange::balanced</v>
@@ -28736,7 +28696,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O62" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P62" t="str">
         <v>flow-state::physical_rhythm_creative_movement_social_exchange_deep_focus::concentrated</v>
@@ -28786,7 +28746,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O63" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P63" t="str">
         <v>flow-state::physical_rhythm_creative_movement_social_exchange_deep_focus::paired</v>
@@ -28836,7 +28796,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O64" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P64" t="str">
         <v>flow-state::physical_rhythm_creative_movement_social_exchange_deep_focus::graduated</v>
@@ -28886,7 +28846,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O65" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P65" t="str">
         <v>flow-state::physical_rhythm_creative_movement_social_exchange_deep_focus::balanced</v>
@@ -28936,7 +28896,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O66" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P66" t="str">
         <v>flow-state::physical_rhythm_social_exchange_deep_focus_creative_movement::concentrated</v>
@@ -28986,7 +28946,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O67" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P67" t="str">
         <v>flow-state::physical_rhythm_social_exchange_deep_focus_creative_movement::paired</v>
@@ -29036,7 +28996,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O68" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P68" t="str">
         <v>flow-state::physical_rhythm_social_exchange_deep_focus_creative_movement::graduated</v>
@@ -29086,7 +29046,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O69" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P69" t="str">
         <v>flow-state::physical_rhythm_social_exchange_deep_focus_creative_movement::balanced</v>
@@ -29136,7 +29096,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O70" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P70" t="str">
         <v>flow-state::physical_rhythm_social_exchange_creative_movement_deep_focus::concentrated</v>
@@ -29186,7 +29146,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O71" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P71" t="str">
         <v>flow-state::physical_rhythm_social_exchange_creative_movement_deep_focus::paired</v>
@@ -29236,7 +29196,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O72" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P72" t="str">
         <v>flow-state::physical_rhythm_social_exchange_creative_movement_deep_focus::graduated</v>
@@ -29286,7 +29246,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O73" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P73" t="str">
         <v>flow-state::physical_rhythm_social_exchange_creative_movement_deep_focus::balanced</v>
@@ -29336,7 +29296,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O74" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P74" t="str">
         <v>flow-state::social_exchange_deep_focus_creative_movement_physical_rhythm::concentrated</v>
@@ -29386,7 +29346,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O75" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P75" t="str">
         <v>flow-state::social_exchange_deep_focus_creative_movement_physical_rhythm::paired</v>
@@ -29436,7 +29396,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O76" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P76" t="str">
         <v>flow-state::social_exchange_deep_focus_creative_movement_physical_rhythm::graduated</v>
@@ -29486,7 +29446,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O77" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P77" t="str">
         <v>flow-state::social_exchange_deep_focus_creative_movement_physical_rhythm::balanced</v>
@@ -29536,7 +29496,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O78" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P78" t="str">
         <v>flow-state::social_exchange_deep_focus_physical_rhythm_creative_movement::concentrated</v>
@@ -29586,7 +29546,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O79" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P79" t="str">
         <v>flow-state::social_exchange_deep_focus_physical_rhythm_creative_movement::paired</v>
@@ -29636,7 +29596,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O80" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P80" t="str">
         <v>flow-state::social_exchange_deep_focus_physical_rhythm_creative_movement::graduated</v>
@@ -29686,7 +29646,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O81" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P81" t="str">
         <v>flow-state::social_exchange_deep_focus_physical_rhythm_creative_movement::balanced</v>
@@ -29736,7 +29696,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O82" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P82" t="str">
         <v>flow-state::social_exchange_creative_movement_deep_focus_physical_rhythm::concentrated</v>
@@ -29786,7 +29746,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O83" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P83" t="str">
         <v>flow-state::social_exchange_creative_movement_deep_focus_physical_rhythm::paired</v>
@@ -29836,7 +29796,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O84" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P84" t="str">
         <v>flow-state::social_exchange_creative_movement_deep_focus_physical_rhythm::graduated</v>
@@ -29886,7 +29846,7 @@
         <v>What to use deliberately: movement, pace, and physical reset.</v>
       </c>
       <c r="O85" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P85" t="str">
         <v>flow-state::social_exchange_creative_movement_deep_focus_physical_rhythm::balanced</v>
@@ -29936,7 +29896,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O86" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P86" t="str">
         <v>flow-state::social_exchange_creative_movement_physical_rhythm_deep_focus::concentrated</v>
@@ -29986,7 +29946,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O87" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P87" t="str">
         <v>flow-state::social_exchange_creative_movement_physical_rhythm_deep_focus::paired</v>
@@ -30036,7 +29996,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O88" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P88" t="str">
         <v>flow-state::social_exchange_creative_movement_physical_rhythm_deep_focus::graduated</v>
@@ -30086,7 +30046,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O89" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P89" t="str">
         <v>flow-state::social_exchange_creative_movement_physical_rhythm_deep_focus::balanced</v>
@@ -30136,7 +30096,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O90" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P90" t="str">
         <v>flow-state::social_exchange_physical_rhythm_deep_focus_creative_movement::concentrated</v>
@@ -30186,7 +30146,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O91" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P91" t="str">
         <v>flow-state::social_exchange_physical_rhythm_deep_focus_creative_movement::paired</v>
@@ -30236,7 +30196,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O92" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P92" t="str">
         <v>flow-state::social_exchange_physical_rhythm_deep_focus_creative_movement::graduated</v>
@@ -30286,7 +30246,7 @@
         <v>What to use deliberately: ideas, expression, and new angles before the work becomes too fixed.</v>
       </c>
       <c r="O93" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P93" t="str">
         <v>flow-state::social_exchange_physical_rhythm_deep_focus_creative_movement::balanced</v>
@@ -30336,7 +30296,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O94" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P94" t="str">
         <v>flow-state::social_exchange_physical_rhythm_creative_movement_deep_focus::concentrated</v>
@@ -30386,7 +30346,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O95" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P95" t="str">
         <v>flow-state::social_exchange_physical_rhythm_creative_movement_deep_focus::paired</v>
@@ -30436,7 +30396,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O96" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P96" t="str">
         <v>flow-state::social_exchange_physical_rhythm_creative_movement_deep_focus::graduated</v>
@@ -30486,7 +30446,7 @@
         <v>What to use deliberately: focused time to finish and refine the work.</v>
       </c>
       <c r="O97" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="P97" t="str">
         <v>flow-state::social_exchange_physical_rhythm_creative_movement_deep_focus::balanced</v>

</xml_diff>

<commit_message>
Fix Flow State preview case status
</commit_message>
<xml_diff>
--- a/content/assessment-packages/flow-state/sonartra_reader_first_import_schema_FLOW_STATE_EXAMPLE.xlsx
+++ b/content/assessment-packages/flow-state/sonartra_reader_first_import_schema_FLOW_STATE_EXAMPLE.xlsx
@@ -19016,7 +19016,7 @@
         <v>context,orientation,recognition,signal_roles,pattern_mechanics,pattern_synthesis,strengths,narrowing,application,closing_integration</v>
       </c>
       <c r="P2" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="Q2" t="str">
         <v>flow-state::preview::concentrated_deep_focus</v>
@@ -19069,7 +19069,7 @@
         <v>context,orientation,recognition,signal_roles,pattern_mechanics,pattern_synthesis,strengths,narrowing,application,closing_integration</v>
       </c>
       <c r="P3" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="Q3" t="str">
         <v>flow-state::preview::paired_deep_focus_creative_movement</v>
@@ -19122,7 +19122,7 @@
         <v>context,orientation,recognition,signal_roles,pattern_mechanics,pattern_synthesis,strengths,narrowing,application,closing_integration</v>
       </c>
       <c r="P4" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="Q4" t="str">
         <v>flow-state::preview::graduated_deep_focus_sequence</v>
@@ -19175,7 +19175,7 @@
         <v>context,orientation,recognition,signal_roles,pattern_mechanics,pattern_synthesis,strengths,narrowing,application,closing_integration</v>
       </c>
       <c r="P5" t="str">
-        <v>draft</v>
+        <v>active</v>
       </c>
       <c r="Q5" t="str">
         <v>flow-state::preview::balanced_deep_focus_sequence</v>

</xml_diff>